<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 20:49 UTC
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2393" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="538">
   <si>
     <t>50001557 - ATACAMA KOZAN</t>
   </si>
@@ -3412,9 +3412,11 @@
       <c r="B23" s="8">
         <v>46168.68298827547</v>
       </c>
-      <c r="C23" s="9"/>
+      <c r="C23" s="8">
+        <v>46197.85300722222</v>
+      </c>
       <c r="D23" s="8">
-        <v>46193.55308</v>
+        <v>46197.85302019676</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>87</v>
@@ -3449,8 +3451,12 @@
       <c r="Q23" s="9"/>
       <c r="R23" s="9"/>
       <c r="S23" s="9"/>
-      <c r="T23" s="9"/>
-      <c r="U23" s="9"/>
+      <c r="T23" s="9">
+        <v>1</v>
+      </c>
+      <c r="U23" s="10" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
@@ -3654,9 +3660,11 @@
       <c r="B27" s="8">
         <v>46168.68321476852</v>
       </c>
-      <c r="C27" s="9"/>
+      <c r="C27" s="8">
+        <v>46197.852991875</v>
+      </c>
       <c r="D27" s="8">
-        <v>46191.16899662037</v>
+        <v>46197.8530077662</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>100</v>
@@ -3704,10 +3712,10 @@
         <v>105</v>
       </c>
       <c r="T27" s="9">
-        <v>0</v>
-      </c>
-      <c r="U27" s="11" t="s">
-        <v>72</v>
+        <v>1</v>
+      </c>
+      <c r="U27" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -4882,7 +4890,7 @@
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="8">
-        <v>46192.17523146991</v>
+        <v>46197.85300241898</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>169</v>
@@ -6955,7 +6963,7 @@
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46168.849797476854</v>
+        <v>46197.851189953704</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>258</v>
@@ -7063,9 +7071,11 @@
       <c r="B86" s="5">
         <v>46168.68352011574</v>
       </c>
-      <c r="C86" s="6"/>
+      <c r="C86" s="5">
+        <v>46197.85117512732</v>
+      </c>
       <c r="D86" s="5">
-        <v>46168.86519618056</v>
+        <v>46197.851191678245</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>266</v>
@@ -7113,10 +7123,10 @@
         <v>32</v>
       </c>
       <c r="T86" s="6">
-        <v>0</v>
-      </c>
-      <c r="U86" s="12" t="s">
-        <v>129</v>
+        <v>1</v>
+      </c>
+      <c r="U86" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -7189,9 +7199,11 @@
       <c r="B88" s="5">
         <v>46168.68353292824</v>
       </c>
-      <c r="C88" s="6"/>
+      <c r="C88" s="5">
+        <v>46197.851300173614</v>
+      </c>
       <c r="D88" s="5">
-        <v>46168.8652724537</v>
+        <v>46197.851317175926</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>273</v>
@@ -7239,10 +7251,10 @@
         <v>32</v>
       </c>
       <c r="T88" s="6">
-        <v>0</v>
-      </c>
-      <c r="U88" s="12" t="s">
-        <v>129</v>
+        <v>1</v>
+      </c>
+      <c r="U88" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -7315,9 +7327,11 @@
       <c r="B90" s="5">
         <v>46168.68354247685</v>
       </c>
-      <c r="C90" s="6"/>
+      <c r="C90" s="5">
+        <v>46197.85161460648</v>
+      </c>
       <c r="D90" s="5">
-        <v>46168.8653077662</v>
+        <v>46197.85163635417</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>277</v>
@@ -7365,10 +7379,10 @@
         <v>32</v>
       </c>
       <c r="T90" s="6">
-        <v>0</v>
-      </c>
-      <c r="U90" s="12" t="s">
-        <v>129</v>
+        <v>1</v>
+      </c>
+      <c r="U90" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
@@ -7380,7 +7394,7 @@
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46192.63406376158</v>
+        <v>46197.85008266204</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>280</v>
@@ -7429,7 +7443,7 @@
         <v>46192.63405665509</v>
       </c>
       <c r="D92" s="5">
-        <v>46192.63407395833</v>
+        <v>46197.85264056713</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>283</v>
@@ -7490,9 +7504,11 @@
       <c r="B93" s="8">
         <v>46168.68356208333</v>
       </c>
-      <c r="C93" s="9"/>
+      <c r="C93" s="8">
+        <v>46197.85262831018</v>
+      </c>
       <c r="D93" s="8">
-        <v>46168.8654994213</v>
+        <v>46197.85263298611</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>213</v>
@@ -7543,9 +7559,11 @@
       <c r="B94" s="5">
         <v>46168.68356922454</v>
       </c>
-      <c r="C94" s="6"/>
+      <c r="C94" s="5">
+        <v>46197.85262942129</v>
+      </c>
       <c r="D94" s="5">
-        <v>46168.865495868056</v>
+        <v>46197.85263334491</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>213</v>
@@ -7596,9 +7614,11 @@
       <c r="B95" s="8">
         <v>46168.683574780094</v>
       </c>
-      <c r="C95" s="9"/>
+      <c r="C95" s="8">
+        <v>46197.85263005787</v>
+      </c>
       <c r="D95" s="8">
-        <v>46168.865493136575</v>
+        <v>46197.85263368055</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>217</v>
@@ -7649,9 +7669,11 @@
       <c r="B96" s="5">
         <v>46168.68358024306</v>
       </c>
-      <c r="C96" s="6"/>
+      <c r="C96" s="5">
+        <v>46197.85263069444</v>
+      </c>
       <c r="D96" s="5">
-        <v>46168.86549053241</v>
+        <v>46197.852634062496</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>217</v>
@@ -7702,9 +7724,11 @@
       <c r="B97" s="8">
         <v>46168.68358578703</v>
       </c>
-      <c r="C97" s="9"/>
+      <c r="C97" s="8">
+        <v>46197.85263130787</v>
+      </c>
       <c r="D97" s="8">
-        <v>46168.86548636574</v>
+        <v>46197.852634490744</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>221</v>
@@ -7755,9 +7779,11 @@
       <c r="B98" s="5">
         <v>46168.68365474537</v>
       </c>
-      <c r="C98" s="6"/>
+      <c r="C98" s="5">
+        <v>46197.85007665509</v>
+      </c>
       <c r="D98" s="5">
-        <v>46168.865691921295</v>
+        <v>46197.85243150463</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>299</v>
@@ -7805,10 +7831,10 @@
         <v>32</v>
       </c>
       <c r="T98" s="6">
-        <v>0</v>
-      </c>
-      <c r="U98" s="12" t="s">
-        <v>129</v>
+        <v>1</v>
+      </c>
+      <c r="U98" s="11" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7818,9 +7844,11 @@
       <c r="B99" s="8">
         <v>46168.683659965274</v>
       </c>
-      <c r="C99" s="9"/>
+      <c r="C99" s="8">
+        <v>46197.85183020833</v>
+      </c>
       <c r="D99" s="8">
-        <v>46190.60542900463</v>
+        <v>46197.852639861114</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>213</v>
@@ -7871,9 +7899,11 @@
       <c r="B100" s="5">
         <v>46168.68366613426</v>
       </c>
-      <c r="C100" s="6"/>
+      <c r="C100" s="5">
+        <v>46197.85205292824</v>
+      </c>
       <c r="D100" s="5">
-        <v>46190.605429560186</v>
+        <v>46197.85263996528</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>213</v>
@@ -7924,9 +7954,11 @@
       <c r="B101" s="8">
         <v>46168.683671921295</v>
       </c>
-      <c r="C101" s="9"/>
+      <c r="C101" s="8">
+        <v>46197.852225717594</v>
+      </c>
       <c r="D101" s="8">
-        <v>46168.8656500463</v>
+        <v>46197.852640173616</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>217</v>
@@ -7977,9 +8009,11 @@
       <c r="B102" s="5">
         <v>46168.68367622685</v>
       </c>
-      <c r="C102" s="6"/>
+      <c r="C102" s="5">
+        <v>46197.8523160301</v>
+      </c>
       <c r="D102" s="5">
-        <v>46168.8656471412</v>
+        <v>46197.85264196759</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>217</v>
@@ -8030,9 +8064,11 @@
       <c r="B103" s="8">
         <v>46168.683680069444</v>
       </c>
-      <c r="C103" s="9"/>
+      <c r="C103" s="8">
+        <v>46197.852413217595</v>
+      </c>
       <c r="D103" s="8">
-        <v>46168.865643125</v>
+        <v>46197.85264373843</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>221</v>
@@ -8148,7 +8184,7 @@
       </c>
       <c r="C105" s="9"/>
       <c r="D105" s="8">
-        <v>46190.60544303241</v>
+        <v>46197.85183748843</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>213</v>
@@ -8201,7 +8237,7 @@
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46190.60543011574</v>
+        <v>46197.852060370366</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>318</v>
@@ -8254,7 +8290,7 @@
       </c>
       <c r="C107" s="9"/>
       <c r="D107" s="8">
-        <v>46168.86584442129</v>
+        <v>46197.85223857639</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>217</v>
@@ -8307,7 +8343,7 @@
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46168.86584158565</v>
+        <v>46197.85232365741</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>217</v>
@@ -8360,7 +8396,7 @@
       </c>
       <c r="C109" s="9"/>
       <c r="D109" s="8">
-        <v>46168.865837881945</v>
+        <v>46197.85242358796</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>221</v>
@@ -8989,7 +9025,7 @@
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46168.86612511574</v>
+        <v>46197.85223737269</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>217</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-01 15:04 UTC
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
@@ -5189,7 +5189,7 @@
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46169.88071780093</v>
+        <v>46204.601559456016</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>182</v>
@@ -5239,8 +5239,8 @@
       <c r="T52" s="6">
         <v>0</v>
       </c>
-      <c r="U52" s="12" t="s">
-        <v>129</v>
+      <c r="U52" s="11" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -5250,9 +5250,11 @@
       <c r="B53" s="8">
         <v>46168.68337377315</v>
       </c>
-      <c r="C53" s="9"/>
+      <c r="C53" s="8">
+        <v>46204.601483715276</v>
+      </c>
       <c r="D53" s="8">
-        <v>46199.1706862963</v>
+        <v>46204.601485555555</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>114</v>
@@ -5303,9 +5305,11 @@
       <c r="B54" s="5">
         <v>46168.683378194444</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46204.60153940972</v>
+      </c>
       <c r="D54" s="5">
-        <v>46169.880830787035</v>
+        <v>46204.601540787036</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>189</v>
@@ -5358,7 +5362,7 @@
       </c>
       <c r="C55" s="9"/>
       <c r="D55" s="8">
-        <v>46169.88084712963</v>
+        <v>46204.60155028936</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>192</v>
@@ -8701,7 +8705,7 @@
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46168.866013425926</v>
+        <v>46204.60155983796</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>337</v>
@@ -8751,8 +8755,8 @@
       <c r="T114" s="6">
         <v>0</v>
       </c>
-      <c r="U114" s="12" t="s">
-        <v>129</v>
+      <c r="U114" s="11" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-02 16:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
@@ -5374,9 +5374,11 @@
       <c r="B55" s="8">
         <v>46168.68338271991</v>
       </c>
-      <c r="C55" s="9"/>
+      <c r="C55" s="8">
+        <v>46205.64435017361</v>
+      </c>
       <c r="D55" s="8">
-        <v>46204.60155028936</v>
+        <v>46205.644352627314</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>192</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-08 20:22 UTC
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
@@ -6673,9 +6673,11 @@
       <c r="B78" s="5">
         <v>46168.683480625</v>
       </c>
-      <c r="C78" s="6"/>
+      <c r="C78" s="5">
+        <v>46211.83846215278</v>
+      </c>
       <c r="D78" s="5">
-        <v>46168.86495055555</v>
+        <v>46211.83847391204</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>246</v>
@@ -6721,10 +6723,10 @@
         <v>32</v>
       </c>
       <c r="T78" s="6">
-        <v>0</v>
-      </c>
-      <c r="U78" s="12" t="s">
-        <v>129</v>
+        <v>1</v>
+      </c>
+      <c r="U78" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6734,9 +6736,11 @@
       <c r="B79" s="8">
         <v>46168.683484629626</v>
       </c>
-      <c r="C79" s="9"/>
+      <c r="C79" s="8">
+        <v>46211.83842483796</v>
+      </c>
       <c r="D79" s="8">
-        <v>46206.48580733796</v>
+        <v>46211.83842664352</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>212</v>
@@ -6787,9 +6791,11 @@
       <c r="B80" s="5">
         <v>46168.683488877316</v>
       </c>
-      <c r="C80" s="6"/>
+      <c r="C80" s="5">
+        <v>46211.83843038195</v>
+      </c>
       <c r="D80" s="5">
-        <v>46206.48579508102</v>
+        <v>46211.83843200232</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>212</v>
@@ -6840,9 +6846,11 @@
       <c r="B81" s="8">
         <v>46168.68349300926</v>
       </c>
-      <c r="C81" s="9"/>
+      <c r="C81" s="8">
+        <v>46211.83843398148</v>
+      </c>
       <c r="D81" s="8">
-        <v>46206.48578787037</v>
+        <v>46211.83843496528</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>216</v>
@@ -6893,9 +6901,11 @@
       <c r="B82" s="5">
         <v>46168.6834959375</v>
       </c>
-      <c r="C82" s="6"/>
+      <c r="C82" s="5">
+        <v>46211.83843877315</v>
+      </c>
       <c r="D82" s="5">
-        <v>46206.48578125</v>
+        <v>46211.83844040509</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>216</v>
@@ -6946,9 +6956,11 @@
       <c r="B83" s="8">
         <v>46168.68349899305</v>
       </c>
-      <c r="C83" s="9"/>
+      <c r="C83" s="8">
+        <v>46211.838444583336</v>
+      </c>
       <c r="D83" s="8">
-        <v>46204.89334085648</v>
+        <v>46211.83844619213</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>220</v>
@@ -10709,7 +10721,7 @@
         <v>46206.48597313657</v>
       </c>
       <c r="D148" s="5">
-        <v>46206.48597475694</v>
+        <v>46211.838432476856</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>212</v>
@@ -10764,7 +10776,7 @@
         <v>46206.48603997685</v>
       </c>
       <c r="D149" s="8">
-        <v>46206.48604142361</v>
+        <v>46211.83844157407</v>
       </c>
       <c r="E149" s="9" t="s">
         <v>212</v>
@@ -10819,7 +10831,7 @@
         <v>46206.48609505787</v>
       </c>
       <c r="D150" s="5">
-        <v>46206.48609666667</v>
+        <v>46211.83843866899</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>216</v>
@@ -10874,7 +10886,7 @@
         <v>46206.48614579861</v>
       </c>
       <c r="D151" s="8">
-        <v>46206.48614756945</v>
+        <v>46211.83844565973</v>
       </c>
       <c r="E151" s="9" t="s">
         <v>216</v>
@@ -10929,7 +10941,7 @@
         <v>46206.48619949074</v>
       </c>
       <c r="D152" s="5">
-        <v>46206.4862009375</v>
+        <v>46211.83845115741</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>220</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-16 09:44 Chile
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4335-4337-4339.xlsx
@@ -2804,7 +2804,7 @@
         <v>46196.89414587963</v>
       </c>
       <c r="D12" s="5">
-        <v>46228.17456038194</v>
+        <v>46249.93870108796</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>56</v>
@@ -4018,7 +4018,7 @@
         <v>46205.61593267361</v>
       </c>
       <c r="D32" s="5">
-        <v>46205.61594793982</v>
+        <v>46249.98766475695</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>118</v>
@@ -6708,7 +6708,7 @@
         <v>46211.83846215278</v>
       </c>
       <c r="D78" s="5">
-        <v>46239.194167118054</v>
+        <v>46249.940088206014</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>245</v>
@@ -7489,7 +7489,7 @@
         <v>46211.83132788194</v>
       </c>
       <c r="D91" s="8">
-        <v>46211.83134737269</v>
+        <v>46249.99091736111</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>278</v>
@@ -7542,7 +7542,7 @@
         <v>46192.63405665509</v>
       </c>
       <c r="D92" s="5">
-        <v>46244.91622329861</v>
+        <v>46249.94030350694</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>281</v>
@@ -7882,7 +7882,7 @@
         <v>46197.85007665509</v>
       </c>
       <c r="D98" s="5">
-        <v>46224.175157731486</v>
+        <v>46249.940361388886</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>297</v>
@@ -8222,7 +8222,7 @@
         <v>46204.89009226851</v>
       </c>
       <c r="D104" s="5">
-        <v>46225.167433888884</v>
+        <v>46249.94047336806</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>311</v>
@@ -8991,7 +8991,7 @@
         <v>46204.89075866898</v>
       </c>
       <c r="D117" s="8">
-        <v>46232.183549988426</v>
+        <v>46249.94056688657</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>343</v>
@@ -9331,7 +9331,7 @@
         <v>46204.89175555555</v>
       </c>
       <c r="D123" s="8">
-        <v>46233.16842686343</v>
+        <v>46249.94067694445</v>
       </c>
       <c r="E123" s="9" t="s">
         <v>355</v>
@@ -9671,7 +9671,7 @@
         <v>46204.89298883102</v>
       </c>
       <c r="D129" s="8">
-        <v>46234.18465609953</v>
+        <v>46249.940871412036</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>370</v>
@@ -10011,7 +10011,7 @@
         <v>46204.893422152774</v>
       </c>
       <c r="D135" s="8">
-        <v>46235.16899013889</v>
+        <v>46249.94102355324</v>
       </c>
       <c r="E135" s="9" t="s">
         <v>385</v>
@@ -10351,7 +10351,7 @@
         <v>46206.4858124537</v>
       </c>
       <c r="D141" s="8">
-        <v>46238.20125695602</v>
+        <v>46249.941063645834</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>399</v>
@@ -10691,7 +10691,7 @@
         <v>46206.48621289352</v>
       </c>
       <c r="D147" s="8">
-        <v>46240.20595440972</v>
+        <v>46249.94115042824</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>410</v>
@@ -11031,7 +11031,7 @@
         <v>46211.8327128588</v>
       </c>
       <c r="D153" s="8">
-        <v>46211.832724733795</v>
+        <v>46249.98997956018</v>
       </c>
       <c r="E153" s="9" t="s">
         <v>422</v>
@@ -11084,7 +11084,7 @@
         <v>46211.83269833333</v>
       </c>
       <c r="D154" s="5">
-        <v>46241.168156099535</v>
+        <v>46249.94153305556</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>425</v>
@@ -11754,7 +11754,7 @@
         <v>46211.83055506945</v>
       </c>
       <c r="D166" s="5">
-        <v>46242.18564827547</v>
+        <v>46249.941719131944</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>447</v>
@@ -12400,7 +12400,7 @@
         <v>46209.71534268519</v>
       </c>
       <c r="D178" s="5">
-        <v>46245.173739502316</v>
+        <v>46249.94202814814</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>468</v>
@@ -13068,7 +13068,7 @@
         <v>46211.83022659722</v>
       </c>
       <c r="D190" s="5">
-        <v>46246.198753125005</v>
+        <v>46249.94212266203</v>
       </c>
       <c r="E190" s="6" t="s">
         <v>494</v>

</xml_diff>